<commit_message>
feat: add description to QuantitativeValue
</commit_message>
<xml_diff>
--- a/HealthRI Imaging metadata model v0.1.0.xlsx
+++ b/HealthRI Imaging metadata model v0.1.0.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alexanderharms/Documents/Projects/Imaging-Metadata-Petal/health-ri-metadata-imaging/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C942A603-AAC6-F248-9147-7AD2247B1132}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69DDB0E4-2784-6E48-98C8-D0D169E52E37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34400" yWindow="-28200" windowWidth="34400" windowHeight="26380" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34400" yWindow="-28200" windowWidth="34400" windowHeight="26380" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="14" r:id="rId1"/>
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="599" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="600" uniqueCount="265">
   <si>
     <t>Property label</t>
   </si>
@@ -855,6 +855,9 @@
   </si>
   <si>
     <t>schema:Number</t>
+  </si>
+  <si>
+    <t>Object to display the minimum and maximum value of a property.</t>
   </si>
 </sst>
 </file>
@@ -5941,12 +5944,15 @@
         <v>105</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>155</v>
       </c>
       <c r="B12" t="s">
         <v>157</v>
+      </c>
+      <c r="C12" s="37" t="s">
+        <v>264</v>
       </c>
       <c r="D12" t="s">
         <v>156</v>

</xml_diff>

<commit_message>
docs: adds description of new classes, adds metadata queries
</commit_message>
<xml_diff>
--- a/HealthRI Imaging metadata model v0.1.0.xlsx
+++ b/HealthRI Imaging metadata model v0.1.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alexanderharms/Documents/Projects/Imaging-Metadata-Petal/health-ri-metadata-imaging/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69DDB0E4-2784-6E48-98C8-D0D169E52E37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B62D47A-D5EF-B94D-881C-060162AC2FCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="34400" yWindow="-28200" windowWidth="34400" windowHeight="26380" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -488,9 +488,6 @@
     <t>SIO.SIO_000999</t>
   </si>
   <si>
-    <t>An ImagingSessionProtocol describes a protocol used for creating the imaging sessions in this dataset. An imaging session is defined as an event which clinically would result in one report. An imaging session consists of one or more scans.</t>
-  </si>
-  <si>
     <t>CTImagingSessionProtocol</t>
   </si>
   <si>
@@ -518,9 +515,6 @@
     <t>hri:ScanProtocol</t>
   </si>
   <si>
-    <t>ScanProtocol describes the protocol used for one or multiple acquisitions (slices) using the same parameters on a patient, as part of an imaging session.</t>
-  </si>
-  <si>
     <t>An ScanProtocol for CT imaging.</t>
   </si>
   <si>
@@ -858,6 +852,12 @@
   </si>
   <si>
     <t>Object to display the minimum and maximum value of a property.</t>
+  </si>
+  <si>
+    <t>An ImagingSessionProtocol describes a protocol used for creating the imaging sessions in this dataset. An imaging session is defined as an event which clinically would result in one report. An imaging session consists of one or more scans. This corresponds to the level of a DICOM Study.</t>
+  </si>
+  <si>
+    <t>ScanProtocol describes the protocol used for one or multiple acquisitions (slices) using the same parameters on a patient, as part of an imaging session. This corresponds to the level of a DICOM Series.</t>
   </si>
 </sst>
 </file>
@@ -3930,7 +3930,7 @@
         <v>7</v>
       </c>
       <c r="I1" s="21" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="J1" s="23" t="s">
         <v>8</v>
@@ -3965,23 +3965,23 @@
     </row>
     <row r="2" spans="1:19" s="24" customFormat="1" ht="64" x14ac:dyDescent="0.2">
       <c r="A2" s="39" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B2" s="39" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D2" s="41"/>
       <c r="E2" s="28" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F2" s="27" t="s">
         <v>9</v>
       </c>
       <c r="G2" s="41" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="H2" s="39" t="s">
         <v>14</v>
@@ -4000,16 +4000,16 @@
     </row>
     <row r="3" spans="1:19" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="39" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B3" s="39" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="F3" s="27" t="s">
         <v>9</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="H3" s="39">
         <v>1</v>
@@ -4020,7 +4020,7 @@
         <v>15</v>
       </c>
       <c r="B4" s="39" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>16</v>
@@ -4037,13 +4037,13 @@
     </row>
     <row r="5" spans="1:19" ht="48" x14ac:dyDescent="0.2">
       <c r="A5" s="39" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="B5" s="39" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="F5" s="27" t="s">
         <v>12</v>
@@ -4054,16 +4054,16 @@
     </row>
     <row r="6" spans="1:19" ht="48" x14ac:dyDescent="0.2">
       <c r="A6" s="39" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B6" s="39" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="F6" s="27" t="s">
         <v>12</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="H6" s="39" t="s">
         <v>19</v>
@@ -4071,16 +4071,16 @@
     </row>
     <row r="7" spans="1:19" ht="64" x14ac:dyDescent="0.2">
       <c r="A7" s="39" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B7" s="39" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="F7" s="27" t="s">
         <v>12</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="H7" s="39" t="s">
         <v>19</v>
@@ -4088,16 +4088,16 @@
     </row>
     <row r="8" spans="1:19" ht="48" x14ac:dyDescent="0.2">
       <c r="A8" s="42" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B8" s="39" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="F8" s="27" t="s">
         <v>12</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="H8" s="42" t="s">
         <v>19</v>
@@ -4105,16 +4105,16 @@
     </row>
     <row r="9" spans="1:19" ht="48" x14ac:dyDescent="0.2">
       <c r="A9" s="39" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="B9" s="39" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="F9" s="27" t="s">
         <v>12</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="H9" s="39" t="s">
         <v>19</v>
@@ -4122,16 +4122,16 @@
     </row>
     <row r="10" spans="1:19" ht="32" x14ac:dyDescent="0.2">
       <c r="A10" s="39" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B10" s="39" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="F10" s="27" t="s">
         <v>12</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="H10" s="39" t="s">
         <v>19</v>
@@ -4139,16 +4139,16 @@
     </row>
     <row r="11" spans="1:19" ht="64" x14ac:dyDescent="0.2">
       <c r="A11" s="42" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B11" s="39" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="F11" s="27" t="s">
         <v>12</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="H11" s="39" t="s">
         <v>19</v>
@@ -4156,16 +4156,16 @@
     </row>
     <row r="12" spans="1:19" ht="64" x14ac:dyDescent="0.2">
       <c r="A12" s="39" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="B12" s="33" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="F12" s="27" t="s">
         <v>12</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="H12" s="39" t="s">
         <v>19</v>
@@ -4173,16 +4173,16 @@
     </row>
     <row r="13" spans="1:19" ht="64" x14ac:dyDescent="0.2">
       <c r="A13" s="39" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B13" s="33" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="F13" s="27" t="s">
         <v>12</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="H13" s="39" t="s">
         <v>19</v>
@@ -4297,7 +4297,7 @@
         <v>7</v>
       </c>
       <c r="I1" s="21" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="J1" s="23" t="s">
         <v>8</v>
@@ -4332,15 +4332,15 @@
     </row>
     <row r="2" spans="1:19" s="24" customFormat="1" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" s="39" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B2" s="34" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="C2" s="26"/>
       <c r="D2" s="28"/>
       <c r="E2" s="28" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="F2" s="27" t="s">
         <v>9</v>
@@ -4363,10 +4363,10 @@
     </row>
     <row r="3" spans="1:19" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="39" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B3" s="34" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="F3" s="27" t="s">
         <v>9</v>
@@ -4377,16 +4377,16 @@
     </row>
     <row r="4" spans="1:19" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="39" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B4" s="39" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="F4" s="27" t="s">
         <v>12</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>19</v>
@@ -4394,16 +4394,16 @@
     </row>
     <row r="5" spans="1:19" ht="32" x14ac:dyDescent="0.2">
       <c r="A5" s="39" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="B5" s="39" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="F5" s="27" t="s">
         <v>12</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="H5" s="3" t="s">
         <v>19</v>
@@ -4526,7 +4526,7 @@
         <v>7</v>
       </c>
       <c r="I1" s="21" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="J1" s="23" t="s">
         <v>8</v>
@@ -4561,15 +4561,15 @@
     </row>
     <row r="2" spans="1:19" s="25" customFormat="1" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" s="39" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="B2" s="34" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="C2" s="29"/>
       <c r="D2" s="30"/>
       <c r="E2" s="28" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="F2" s="27" t="s">
         <v>9</v>
@@ -4592,16 +4592,16 @@
     </row>
     <row r="3" spans="1:19" ht="48" x14ac:dyDescent="0.2">
       <c r="A3" s="39" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B3" s="44" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="F3" s="27" t="s">
         <v>12</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="H3" s="3" t="s">
         <v>19</v>
@@ -4609,16 +4609,16 @@
     </row>
     <row r="4" spans="1:19" ht="48" x14ac:dyDescent="0.2">
       <c r="A4" s="39" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B4" s="44" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="F4" s="27" t="s">
         <v>12</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>19</v>
@@ -4741,7 +4741,7 @@
         <v>7</v>
       </c>
       <c r="I1" s="21" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="J1" s="23" t="s">
         <v>8</v>
@@ -4776,10 +4776,10 @@
     </row>
     <row r="2" spans="1:19" s="24" customFormat="1" ht="64" x14ac:dyDescent="0.2">
       <c r="A2" s="39" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B2" s="39" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="C2" s="26"/>
       <c r="D2" s="28"/>
@@ -4788,7 +4788,7 @@
         <v>12</v>
       </c>
       <c r="G2" s="27" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="H2" s="27" t="s">
         <v>19</v>
@@ -4807,16 +4807,16 @@
     </row>
     <row r="3" spans="1:19" ht="96" x14ac:dyDescent="0.2">
       <c r="A3" s="39" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B3" s="39" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="F3" s="27" t="s">
         <v>12</v>
       </c>
       <c r="G3" s="27" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="H3" s="3" t="s">
         <v>19</v>
@@ -4939,7 +4939,7 @@
         <v>7</v>
       </c>
       <c r="I1" s="21" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="J1" s="23" t="s">
         <v>8</v>
@@ -5179,7 +5179,7 @@
         <v>7</v>
       </c>
       <c r="I1" s="21" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="J1" s="23" t="s">
         <v>8</v>
@@ -5214,13 +5214,13 @@
     </row>
     <row r="2" spans="1:19" s="24" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="43" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B2" s="39" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="C2" s="39" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="D2" s="28"/>
       <c r="E2" s="28"/>
@@ -5228,7 +5228,7 @@
         <v>9</v>
       </c>
       <c r="G2" s="27" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="H2" s="27">
         <v>1</v>
@@ -5247,19 +5247,19 @@
     </row>
     <row r="3" spans="1:19" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B3" s="39" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="C3" s="39" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="F3" s="27" t="s">
         <v>9</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="H3" s="3">
         <v>1</v>
@@ -5657,18 +5657,18 @@
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B40" s="36" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B41" s="36" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -5773,7 +5773,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="64" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" ht="80" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>135</v>
       </c>
@@ -5781,7 +5781,7 @@
         <v>136</v>
       </c>
       <c r="C3" s="37" t="s">
-        <v>141</v>
+        <v>263</v>
       </c>
       <c r="D3" s="36" t="s">
         <v>139</v>
@@ -5792,13 +5792,13 @@
     </row>
     <row r="4" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>141</v>
+      </c>
+      <c r="B4" t="s">
         <v>142</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" s="37" t="s">
         <v>143</v>
-      </c>
-      <c r="C4" s="37" t="s">
-        <v>144</v>
       </c>
       <c r="D4" s="36" t="s">
         <v>139</v>
@@ -5812,13 +5812,13 @@
     </row>
     <row r="5" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B5" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C5" s="37" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D5" s="36" t="s">
         <v>139</v>
@@ -5832,13 +5832,13 @@
     </row>
     <row r="6" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>145</v>
+      </c>
+      <c r="B6" t="s">
         <v>146</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" s="37" t="s">
         <v>147</v>
-      </c>
-      <c r="C6" s="37" t="s">
-        <v>148</v>
       </c>
       <c r="D6" s="36" t="s">
         <v>139</v>
@@ -5850,15 +5850,15 @@
         <v>140</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" ht="64" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>148</v>
+      </c>
+      <c r="B7" t="s">
         <v>149</v>
       </c>
-      <c r="B7" t="s">
-        <v>150</v>
-      </c>
       <c r="C7" s="37" t="s">
-        <v>151</v>
+        <v>264</v>
       </c>
       <c r="D7" s="36" t="s">
         <v>139</v>
@@ -5869,19 +5869,19 @@
     </row>
     <row r="8" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B8" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C8" s="37" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D8" s="36" t="s">
         <v>139</v>
       </c>
       <c r="E8" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H8" t="s">
         <v>140</v>
@@ -5889,19 +5889,19 @@
     </row>
     <row r="9" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B9" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C9" s="37" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D9" s="36" t="s">
         <v>139</v>
       </c>
       <c r="E9" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H9" t="s">
         <v>140</v>
@@ -5909,19 +5909,19 @@
     </row>
     <row r="10" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B10" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C10" s="37" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="D10" s="36" t="s">
         <v>139</v>
       </c>
       <c r="E10" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H10" t="s">
         <v>140</v>
@@ -5946,19 +5946,19 @@
     </row>
     <row r="12" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
+        <v>153</v>
+      </c>
+      <c r="B12" t="s">
         <v>155</v>
       </c>
-      <c r="B12" t="s">
-        <v>157</v>
-      </c>
       <c r="C12" s="37" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="D12" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="H12" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
   </sheetData>
@@ -5973,6 +5973,7 @@
     <hyperlink ref="D10" r:id="rId8" display="http://semanticscience.org/resource/SIO_000999" xr:uid="{F4839171-3961-FD48-9C84-220699602213}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
@@ -6030,7 +6031,7 @@
         <v>7</v>
       </c>
       <c r="I1" s="21" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="J1" s="23" t="s">
         <v>8</v>
@@ -6065,23 +6066,23 @@
     </row>
     <row r="2" spans="1:19" s="24" customFormat="1" ht="48" x14ac:dyDescent="0.2">
       <c r="A2" s="39" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B2" s="39" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C2" s="26" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="D2" s="40"/>
       <c r="E2" s="28" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="F2" s="27" t="s">
         <v>9</v>
       </c>
       <c r="G2" s="40" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="H2" s="27" t="s">
         <v>14</v>
@@ -6100,23 +6101,23 @@
     </row>
     <row r="3" spans="1:19" ht="48" x14ac:dyDescent="0.2">
       <c r="A3" s="39" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B3" s="39" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="D3" s="41"/>
       <c r="E3" s="28" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F3" s="27" t="s">
         <v>9</v>
       </c>
       <c r="G3" s="41" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="H3" s="3" t="s">
         <v>14</v>
@@ -6124,23 +6125,23 @@
     </row>
     <row r="4" spans="1:19" ht="64" x14ac:dyDescent="0.2">
       <c r="A4" s="39" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B4" s="39" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D4" s="41"/>
       <c r="E4" s="28" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F4" s="27" t="s">
         <v>9</v>
       </c>
       <c r="G4" s="41" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>14</v>
@@ -6148,13 +6149,13 @@
     </row>
     <row r="5" spans="1:19" ht="32" x14ac:dyDescent="0.2">
       <c r="A5" s="39" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B5" s="39" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F5" s="27" t="s">
         <v>12</v>
@@ -6291,7 +6292,7 @@
         <v>7</v>
       </c>
       <c r="I1" s="21" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="J1" s="23" t="s">
         <v>8</v>
@@ -6326,23 +6327,23 @@
     </row>
     <row r="2" spans="1:19" s="24" customFormat="1" ht="48" x14ac:dyDescent="0.2">
       <c r="A2" s="39" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B2" s="39" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C2" s="26" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="D2" s="40"/>
       <c r="E2" s="28" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="F2" s="27" t="s">
         <v>9</v>
       </c>
       <c r="G2" s="40" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="H2" s="27">
         <v>1</v>
@@ -6361,10 +6362,10 @@
     </row>
     <row r="3" spans="1:19" ht="32" x14ac:dyDescent="0.2">
       <c r="A3" s="39" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B3" s="39" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="F3" s="27" t="s">
         <v>9</v>
@@ -6381,7 +6382,7 @@
         <v>15</v>
       </c>
       <c r="B4" s="39" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C4" s="39" t="s">
         <v>16</v>
@@ -6398,16 +6399,16 @@
     </row>
     <row r="5" spans="1:19" ht="32" x14ac:dyDescent="0.2">
       <c r="A5" s="39" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B5" s="33" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="F5" s="27" t="s">
         <v>9</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H5" s="3" t="s">
         <v>14</v>
@@ -6415,23 +6416,23 @@
     </row>
     <row r="6" spans="1:19" ht="48" x14ac:dyDescent="0.2">
       <c r="A6" s="39" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B6" s="39" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="D6" s="41"/>
       <c r="E6" s="28" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F6" s="27" t="s">
         <v>12</v>
       </c>
       <c r="G6" s="41" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="H6" s="3" t="s">
         <v>13</v>
@@ -6439,10 +6440,10 @@
     </row>
     <row r="7" spans="1:19" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="42" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B7" s="39" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>24</v>
@@ -6459,10 +6460,10 @@
     </row>
     <row r="8" spans="1:19" ht="32" x14ac:dyDescent="0.2">
       <c r="A8" s="39" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B8" s="39" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="F8" s="27" t="s">
         <v>12</v>
@@ -6476,13 +6477,13 @@
     </row>
     <row r="9" spans="1:19" ht="48" x14ac:dyDescent="0.2">
       <c r="A9" s="39" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B9" s="39" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="F9" s="27" t="s">
         <v>12</v>
@@ -6493,13 +6494,13 @@
     </row>
     <row r="10" spans="1:19" ht="32" x14ac:dyDescent="0.2">
       <c r="A10" s="39" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B10" s="34" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="E10" s="39" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="F10" s="27" t="s">
         <v>12</v>
@@ -6629,7 +6630,7 @@
         <v>7</v>
       </c>
       <c r="I1" s="21" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="J1" s="23" t="s">
         <v>8</v>
@@ -6664,15 +6665,15 @@
     </row>
     <row r="2" spans="1:19" s="24" customFormat="1" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" s="26" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C2" s="26"/>
       <c r="D2" s="28"/>
       <c r="E2" s="39" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="F2" s="27" t="s">
         <v>9</v>
@@ -6810,7 +6811,7 @@
         <v>7</v>
       </c>
       <c r="I1" s="21" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="J1" s="23" t="s">
         <v>8</v>
@@ -6845,10 +6846,10 @@
     </row>
     <row r="2" spans="1:19" s="25" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="39" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B2" s="39" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C2" s="29"/>
       <c r="D2" s="30"/>
@@ -6857,7 +6858,7 @@
         <v>9</v>
       </c>
       <c r="G2" s="27" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="H2" s="27" t="s">
         <v>14</v>
@@ -6876,13 +6877,13 @@
     </row>
     <row r="3" spans="1:19" ht="32" x14ac:dyDescent="0.2">
       <c r="A3" s="39" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B3" s="39" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="E3" s="39" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="F3" s="27" t="s">
         <v>12</v>
@@ -7008,7 +7009,7 @@
         <v>7</v>
       </c>
       <c r="I1" s="21" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="J1" s="23" t="s">
         <v>8</v>
@@ -7043,15 +7044,15 @@
     </row>
     <row r="2" spans="1:19" s="24" customFormat="1" ht="80" x14ac:dyDescent="0.2">
       <c r="A2" s="39" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B2" s="42" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C2" s="26"/>
       <c r="D2" s="28"/>
       <c r="E2" s="28" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="F2" s="27" t="s">
         <v>9</v>

</xml_diff>